<commit_message>
Fix three ticker/listing errors in semiconductor chain Excel
- 沐曦股份: 非上市 → 688802.SH (上交所科创板, listed 2024)
- 摩尔线程: 非上市 → 688795.SH (上交所科创板, listed 2024)
- 洛阳股份 000537.SZ (广宇集团,错误) → 洛阳钼业 603993.SH (Mo/Cu targets)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J9TDaiFCfdBUVQKBmm5e3u
</commit_message>
<xml_diff>
--- a/半导体全产业链标的.xlsx
+++ b/半导体全产业链标的.xlsx
@@ -283,7 +283,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -402,12 +402,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3883,22 +3877,22 @@
       </c>
       <c r="E58" s="17" t="inlineStr">
         <is>
-          <t>洛阳股份</t>
+          <t>洛阳钼业 China Moly</t>
         </is>
       </c>
       <c r="F58" s="18" t="inlineStr">
         <is>
-          <t>000537.SZ</t>
+          <t>603993.SH</t>
         </is>
       </c>
       <c r="G58" s="19" t="inlineStr">
         <is>
-          <t>深交所</t>
+          <t>上交所</t>
         </is>
       </c>
       <c r="H58" s="19" t="inlineStr">
         <is>
-          <t>钼铜靶材</t>
+          <t>钼/铜靶材/有色金属</t>
         </is>
       </c>
       <c r="I58" s="20" t="inlineStr">
@@ -8459,22 +8453,22 @@
       </c>
       <c r="D142" s="36" t="inlineStr">
         <is>
-          <t>GPU架构芯片（非上市）</t>
-        </is>
-      </c>
-      <c r="E142" s="42" t="inlineStr">
+          <t>GPU架构芯片，2024年登陆科创板</t>
+        </is>
+      </c>
+      <c r="E142" s="37" t="inlineStr">
         <is>
           <t>沐曦股份</t>
         </is>
       </c>
-      <c r="F142" s="43" t="inlineStr">
-        <is>
-          <t>非上市</t>
+      <c r="F142" s="38" t="inlineStr">
+        <is>
+          <t>688802.SH</t>
         </is>
       </c>
       <c r="G142" s="39" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>上交所科创板</t>
         </is>
       </c>
       <c r="H142" s="39" t="inlineStr">
@@ -8512,22 +8506,22 @@
       </c>
       <c r="D143" s="36" t="inlineStr">
         <is>
-          <t>GPU芯片（非上市）</t>
-        </is>
-      </c>
-      <c r="E143" s="42" t="inlineStr">
+          <t>GPU芯片，2024年登陆科创板</t>
+        </is>
+      </c>
+      <c r="E143" s="37" t="inlineStr">
         <is>
           <t>摩尔线程</t>
         </is>
       </c>
-      <c r="F143" s="43" t="inlineStr">
-        <is>
-          <t>非上市</t>
+      <c r="F143" s="38" t="inlineStr">
+        <is>
+          <t>688795.SH</t>
         </is>
       </c>
       <c r="G143" s="39" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>上交所科创板</t>
         </is>
       </c>
       <c r="H143" s="39" t="inlineStr">

</xml_diff>

<commit_message>
Add Nebius (NBIS) to 算力租赁 in Stage 5 AI算力
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J9TDaiFCfdBUVQKBmm5e3u
</commit_message>
<xml_diff>
--- a/半导体全产业链标的.xlsx
+++ b/半导体全产业链标的.xlsx
@@ -830,7 +830,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V246"/>
+  <dimension ref="A1:V247"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15610,8 +15610,8 @@
       <c r="V245" s="13" t="inlineStr"/>
     </row>
     <row r="246" ht="16" customHeight="1">
-      <c r="A246" s="16" t="n"/>
-      <c r="B246" s="16" t="n"/>
+      <c r="A246" s="15" t="n"/>
+      <c r="B246" s="15" t="n"/>
       <c r="C246" s="37" t="inlineStr">
         <is>
           <t>AI算力</t>
@@ -15664,6 +15664,62 @@
       <c r="T246" s="13" t="inlineStr"/>
       <c r="U246" s="13" t="inlineStr"/>
       <c r="V246" s="13" t="inlineStr"/>
+    </row>
+    <row r="247" ht="16" customHeight="1">
+      <c r="A247" s="16" t="n"/>
+      <c r="B247" s="16" t="n"/>
+      <c r="C247" s="37" t="inlineStr">
+        <is>
+          <t>AI算力</t>
+        </is>
+      </c>
+      <c r="D247" s="38" t="inlineStr">
+        <is>
+          <t>GPU云算力租赁，欧洲最大AI基础设施云平台，从Yandex拆分上市</t>
+        </is>
+      </c>
+      <c r="E247" s="39" t="inlineStr">
+        <is>
+          <t>Nebius Group</t>
+        </is>
+      </c>
+      <c r="F247" s="40" t="inlineStr">
+        <is>
+          <t>NBIS</t>
+        </is>
+      </c>
+      <c r="G247" s="41" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="H247" s="41" t="inlineStr">
+        <is>
+          <t>GPU云/AI基础设施租赁</t>
+        </is>
+      </c>
+      <c r="I247" s="42" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J247" s="23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K247" s="13" t="inlineStr"/>
+      <c r="L247" s="13" t="inlineStr"/>
+      <c r="M247" s="13" t="inlineStr"/>
+      <c r="N247" s="13" t="inlineStr"/>
+      <c r="O247" s="13" t="inlineStr"/>
+      <c r="P247" s="13" t="inlineStr"/>
+      <c r="Q247" s="13" t="inlineStr"/>
+      <c r="R247" s="13" t="inlineStr"/>
+      <c r="S247" s="13" t="inlineStr"/>
+      <c r="T247" s="13" t="inlineStr"/>
+      <c r="U247" s="13" t="inlineStr"/>
+      <c r="V247" s="13" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:V3"/>
@@ -15689,9 +15745,9 @@
     <mergeCell ref="B132:B133"/>
     <mergeCell ref="B139:B141"/>
     <mergeCell ref="B228:B231"/>
+    <mergeCell ref="A178:A247"/>
     <mergeCell ref="B182:B185"/>
     <mergeCell ref="B151:B156"/>
-    <mergeCell ref="B243:B246"/>
     <mergeCell ref="B200:B204"/>
     <mergeCell ref="B119:B122"/>
     <mergeCell ref="B75:B77"/>
@@ -15711,7 +15767,6 @@
     <mergeCell ref="B99:B100"/>
     <mergeCell ref="B134:B138"/>
     <mergeCell ref="B45:B53"/>
-    <mergeCell ref="A178:A246"/>
     <mergeCell ref="B172:B177"/>
     <mergeCell ref="B186:B189"/>
     <mergeCell ref="B15:B20"/>
@@ -15736,6 +15791,7 @@
     <mergeCell ref="B209:B212"/>
     <mergeCell ref="B125:B126"/>
     <mergeCell ref="B85:B88"/>
+    <mergeCell ref="B243:B247"/>
     <mergeCell ref="B21:B22"/>
     <mergeCell ref="B63:B68"/>
     <mergeCell ref="B221:B224"/>

</xml_diff>